<commit_message>
finalizando o 2 refinamento dos hiperparametros para cada ticker
</commit_message>
<xml_diff>
--- a/dados/aux_data/tabela_hiperparametros_MULT3.xlsx
+++ b/dados/aux_data/tabela_hiperparametros_MULT3.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,37 +424,57 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>val_loss_mse</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>units_1</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>units_2</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>dropout</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>learning_rate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>batch_size</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>l2</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>dense_units</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>n_dense</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>optimizer</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>window_size</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>val_loss</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>units_1</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>units_2</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>dropout</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>learning_rate</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>batch_size</t>
         </is>
       </c>
     </row>
@@ -465,109 +485,39 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>60</v>
+        <v>0.02859515510499477</v>
       </c>
       <c r="C2" t="n">
-        <v>0.03469337895512581</v>
+        <v>128</v>
       </c>
       <c r="D2" t="n">
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="E2" t="n">
-        <v>48</v>
+        <v>0.3861029797453003</v>
       </c>
       <c r="F2" t="n">
-        <v>0.3554707436863301</v>
+        <v>0.000825661479489345</v>
       </c>
       <c r="G2" t="n">
-        <v>0.009415194626014265</v>
+        <v>64</v>
       </c>
       <c r="H2" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MULT3</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+        <v>2.968064156807333e-06</v>
+      </c>
+      <c r="I2" t="n">
+        <v>32</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>RMSprop</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
         <v>90</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.03029380738735199</v>
-      </c>
-      <c r="D3" t="n">
-        <v>64</v>
-      </c>
-      <c r="E3" t="n">
-        <v>32</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.2291245132958113</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.009341225088415676</v>
-      </c>
-      <c r="H3" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>MULT3</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>120</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.02832426503300667</v>
-      </c>
-      <c r="D4" t="n">
-        <v>64</v>
-      </c>
-      <c r="E4" t="n">
-        <v>64</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.306184072097302</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.008948811561232728</v>
-      </c>
-      <c r="H4" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>MULT3</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>180</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.03064398653805256</v>
-      </c>
-      <c r="D5" t="n">
-        <v>32</v>
-      </c>
-      <c r="E5" t="n">
-        <v>48</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.1644269136673398</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.009876254271654783</v>
-      </c>
-      <c r="H5" t="n">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>